<commit_message>
Stockholm duplicate rows accruals removed
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/ACRIa.ST.xlsx
+++ b/data/stx_xlsx/ACRIa.ST.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="262">
   <si>
     <t>Company Fundamentals - Income Statement</t>
   </si>
@@ -462,25 +462,28 @@
     <t>Deferred tax Liability</t>
   </si>
   <si>
+    <t>interest - bearing Liabilities to credit institutions (Do not use)</t>
+  </si>
+  <si>
+    <t>Other interest - bearing liabilities</t>
+  </si>
+  <si>
+    <t>Other Non-Current Liabilities - Total</t>
+  </si>
+  <si>
+    <t>Derivative Liabilities - Hedging - Long-Term</t>
+  </si>
+  <si>
+    <t>Balancing Item - Noncurrent Liabilities</t>
+  </si>
+  <si>
+    <t>Other Provisions/Guarantees</t>
+  </si>
+  <si>
+    <t>Noncurrent Liabilities</t>
+  </si>
+  <si>
     <t>interest - bearing Liabilities to credit institutions</t>
-  </si>
-  <si>
-    <t>Other interest - bearing liabilities</t>
-  </si>
-  <si>
-    <t>Other Non-Current Liabilities - Total</t>
-  </si>
-  <si>
-    <t>Derivative Liabilities - Hedging - Long-Term</t>
-  </si>
-  <si>
-    <t>Balancing Item - Noncurrent Liabilities</t>
-  </si>
-  <si>
-    <t>Other Provisions/Guarantees</t>
-  </si>
-  <si>
-    <t>Noncurrent Liabilities</t>
   </si>
   <si>
     <t>Leverantörsskulder</t>
@@ -927,7 +930,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1002,6 +1005,9 @@
     </xf>
     <xf borderId="3" fillId="0" fontId="6" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -5967,7 +5973,7 @@
       <c r="M57" s="17"/>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="14" t="s">
+      <c r="A58" s="25" t="s">
         <v>147</v>
       </c>
       <c r="B58" s="15">
@@ -6198,7 +6204,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="14" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B66" s="16">
         <v>29.74</v>
@@ -6239,7 +6245,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="14" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B67" s="16">
         <v>9.75</v>
@@ -6280,7 +6286,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="14" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B68" s="17"/>
       <c r="C68" s="17"/>
@@ -6299,7 +6305,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="14" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B69" s="17">
         <v>0.0</v>
@@ -6338,7 +6344,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="14" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B70" s="16">
         <v>2.2</v>
@@ -6379,7 +6385,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B71" s="16">
         <v>14.08</v>
@@ -6420,7 +6426,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="18" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B72" s="20">
         <v>89.83</v>
@@ -6461,7 +6467,7 @@
     </row>
     <row r="73" ht="15.0" customHeight="1">
       <c r="A73" s="18" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B73" s="19">
         <v>515.08</v>
@@ -6502,7 +6508,7 @@
     </row>
     <row r="74" ht="15.0" customHeight="1">
       <c r="A74" s="14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B74" s="17"/>
       <c r="C74" s="17"/>
@@ -6525,7 +6531,7 @@
     </row>
     <row r="75" ht="15.0" customHeight="1">
       <c r="A75" s="18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B75" s="19">
         <v>1126.13</v>
@@ -6566,7 +6572,7 @@
     </row>
     <row r="76" ht="15.0" customHeight="1">
       <c r="A76" s="14" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B76" s="17">
         <v>0.0</v>
@@ -6607,7 +6613,7 @@
     </row>
     <row r="77" ht="15.0" customHeight="1">
       <c r="A77" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B77" s="16">
         <v>43.54</v>
@@ -6648,7 +6654,7 @@
     </row>
     <row r="78" ht="15.0" customHeight="1">
       <c r="A78" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B78" s="16">
         <v>43.54</v>
@@ -6689,7 +6695,7 @@
     </row>
     <row r="79" ht="15.0" customHeight="1">
       <c r="A79" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B79" s="16">
         <v>28.5</v>
@@ -6716,7 +6722,7 @@
     </row>
     <row r="80" ht="15.0" customHeight="1">
       <c r="A80" s="14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B80" s="17">
         <v>0.0</v>
@@ -6743,7 +6749,7 @@
     </row>
     <row r="81" ht="15.0" customHeight="1">
       <c r="A81" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B81" s="16">
         <v>0.65</v>
@@ -6770,7 +6776,7 @@
     </row>
     <row r="82" ht="15.0" customHeight="1">
       <c r="A82" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B82" s="16">
         <v>28.5</v>
@@ -6797,7 +6803,7 @@
     </row>
     <row r="83" ht="15.0" customHeight="1">
       <c r="A83" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B83" s="16">
         <v>15.04</v>
@@ -6838,7 +6844,7 @@
     </row>
     <row r="84" ht="15.0" customHeight="1">
       <c r="A84" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B84" s="17">
         <v>0.0</v>
@@ -6877,7 +6883,7 @@
     </row>
     <row r="85" ht="15.0" customHeight="1">
       <c r="A85" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B85" s="16">
         <v>15.04</v>
@@ -6918,7 +6924,7 @@
     </row>
     <row r="86" ht="15.0" customHeight="1">
       <c r="A86" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B86" s="16">
         <v>0.35</v>
@@ -6959,7 +6965,7 @@
     </row>
     <row r="87" ht="15.0" customHeight="1">
       <c r="A87" s="14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B87" s="16">
         <v>8.0</v>
@@ -7915,7 +7921,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -8171,40 +8177,40 @@
         <v>34</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1" outlineLevel="1">
@@ -8250,7 +8256,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -8308,7 +8314,7 @@
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B20" s="16">
         <v>14.61</v>
@@ -8349,7 +8355,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B21" s="21">
         <v>-7.44</v>
@@ -8384,7 +8390,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B22" s="16">
         <v>25.63</v>
@@ -8398,7 +8404,7 @@
       <c r="E22" s="21">
         <v>-44.69</v>
       </c>
-      <c r="F22" s="25">
+      <c r="F22" s="26">
         <v>-150.31</v>
       </c>
       <c r="G22" s="21">
@@ -8425,7 +8431,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B23" s="17"/>
       <c r="C23" s="16">
@@ -8448,7 +8454,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B24" s="17"/>
       <c r="C24" s="17">
@@ -8471,7 +8477,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="17">
@@ -8494,7 +8500,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="21">
@@ -8517,7 +8523,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="14" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
@@ -8536,7 +8542,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="14" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -8555,9 +8561,9 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="B29" s="25">
+        <v>186</v>
+      </c>
+      <c r="B29" s="26">
         <v>-228.61</v>
       </c>
       <c r="C29" s="16">
@@ -8596,7 +8602,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B30" s="15">
         <v>553.52</v>
@@ -8635,7 +8641,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="14" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
@@ -8654,7 +8660,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="14" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="17"/>
@@ -8673,7 +8679,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="18" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B33" s="19">
         <v>357.71</v>
@@ -8714,7 +8720,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="14" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B34" s="15">
         <v>347.08</v>
@@ -8751,7 +8757,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="14" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B35" s="21">
         <v>-23.95</v>
@@ -8772,7 +8778,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="14" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B36" s="21">
         <v>-91.62</v>
@@ -8780,19 +8786,19 @@
       <c r="C36" s="21">
         <v>-49.35</v>
       </c>
-      <c r="D36" s="25">
+      <c r="D36" s="26">
         <v>-148.21</v>
       </c>
       <c r="E36" s="21">
         <v>-75.06</v>
       </c>
-      <c r="F36" s="25">
+      <c r="F36" s="26">
         <v>-608.7</v>
       </c>
-      <c r="G36" s="25">
+      <c r="G36" s="26">
         <v>-210.09</v>
       </c>
-      <c r="H36" s="25">
+      <c r="H36" s="26">
         <v>-210.12</v>
       </c>
       <c r="I36" s="21">
@@ -8801,7 +8807,7 @@
       <c r="J36" s="21">
         <v>-92.74</v>
       </c>
-      <c r="K36" s="25">
+      <c r="K36" s="26">
         <v>-226.1</v>
       </c>
       <c r="L36" s="21">
@@ -8813,7 +8819,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="14" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B37" s="17"/>
       <c r="C37" s="17">
@@ -8850,14 +8856,14 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="14" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B38" s="17"/>
       <c r="C38" s="21">
         <v>-0.48</v>
       </c>
       <c r="D38" s="17"/>
-      <c r="E38" s="25">
+      <c r="E38" s="26">
         <v>-250.41</v>
       </c>
       <c r="F38" s="21">
@@ -8881,7 +8887,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="14" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -8910,7 +8916,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="14" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B40" s="17"/>
       <c r="C40" s="17"/>
@@ -8933,7 +8939,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="18" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B41" s="19">
         <v>231.51</v>
@@ -8941,19 +8947,19 @@
       <c r="C41" s="22">
         <v>-89.25</v>
       </c>
-      <c r="D41" s="26">
+      <c r="D41" s="27">
         <v>-148.83</v>
       </c>
-      <c r="E41" s="26">
+      <c r="E41" s="27">
         <v>-202.27</v>
       </c>
-      <c r="F41" s="26">
+      <c r="F41" s="27">
         <v>-636.52</v>
       </c>
-      <c r="G41" s="26">
+      <c r="G41" s="27">
         <v>-191.22</v>
       </c>
-      <c r="H41" s="26">
+      <c r="H41" s="27">
         <v>-173.17</v>
       </c>
       <c r="I41" s="22">
@@ -8962,7 +8968,7 @@
       <c r="J41" s="22">
         <v>-54.41</v>
       </c>
-      <c r="K41" s="26">
+      <c r="K41" s="27">
         <v>-319.07</v>
       </c>
       <c r="L41" s="20">
@@ -8974,7 +8980,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="14" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
@@ -9007,7 +9013,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="14" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B43" s="15">
         <v>110.93</v>
@@ -9044,12 +9050,12 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="14" t="s">
-        <v>200</v>
-      </c>
-      <c r="B44" s="25">
+        <v>201</v>
+      </c>
+      <c r="B44" s="26">
         <v>-132.98</v>
       </c>
-      <c r="C44" s="25">
+      <c r="C44" s="26">
         <v>-324.53</v>
       </c>
       <c r="D44" s="21">
@@ -9069,7 +9075,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="14" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B45" s="21">
         <v>-1.94</v>
@@ -9090,9 +9096,9 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="14" t="s">
-        <v>202</v>
-      </c>
-      <c r="B46" s="25">
+        <v>203</v>
+      </c>
+      <c r="B46" s="26">
         <v>-101.67</v>
       </c>
       <c r="C46" s="21">
@@ -9131,9 +9137,9 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="14" t="s">
-        <v>203</v>
-      </c>
-      <c r="B47" s="25">
+        <v>204</v>
+      </c>
+      <c r="B47" s="26">
         <v>-389.16</v>
       </c>
       <c r="C47" s="17">
@@ -9156,7 +9162,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B48" s="17"/>
       <c r="C48" s="17"/>
@@ -9175,7 +9181,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="14" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B49" s="17"/>
       <c r="C49" s="17"/>
@@ -9194,7 +9200,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="14" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B50" s="17"/>
       <c r="C50" s="17"/>
@@ -9215,9 +9221,9 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="B51" s="26">
+        <v>208</v>
+      </c>
+      <c r="B51" s="27">
         <v>-514.83</v>
       </c>
       <c r="C51" s="20">
@@ -9256,7 +9262,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="14" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B52" s="16">
         <v>88.73</v>
@@ -9297,7 +9303,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="14" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B53" s="15">
         <v>165.54</v>
@@ -9338,7 +9344,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="14" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B54" s="17"/>
       <c r="C54" s="17"/>
@@ -9359,7 +9365,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="18" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B55" s="20">
         <v>74.39</v>
@@ -10365,7 +10371,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -10681,7 +10687,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -10734,1286 +10740,1286 @@
       </c>
     </row>
     <row r="20" ht="15.0" customHeight="1">
-      <c r="A20" s="27" t="s">
-        <v>214</v>
-      </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="28"/>
+      <c r="A20" s="28" t="s">
+        <v>215</v>
+      </c>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="29"/>
+      <c r="L20" s="29"/>
     </row>
     <row r="21" ht="15.0" customHeight="1">
-      <c r="A21" s="29" t="s">
-        <v>214</v>
-      </c>
-      <c r="B21" s="30">
+      <c r="A21" s="30" t="s">
+        <v>215</v>
+      </c>
+      <c r="B21" s="31">
         <v>1689.47</v>
       </c>
-      <c r="C21" s="30">
+      <c r="C21" s="31">
         <v>1628.99</v>
       </c>
-      <c r="D21" s="30">
+      <c r="D21" s="31">
         <v>1387.62</v>
       </c>
-      <c r="E21" s="30">
+      <c r="E21" s="31">
         <v>1480.46</v>
       </c>
-      <c r="F21" s="30">
+      <c r="F21" s="31">
         <v>569.89</v>
       </c>
-      <c r="G21" s="30">
+      <c r="G21" s="31">
         <v>378.62</v>
       </c>
-      <c r="H21" s="30">
+      <c r="H21" s="31">
         <v>271.09</v>
       </c>
-      <c r="I21" s="30">
+      <c r="I21" s="31">
         <v>248.88</v>
       </c>
-      <c r="J21" s="30">
+      <c r="J21" s="31">
         <v>209.49</v>
       </c>
-      <c r="K21" s="31">
+      <c r="K21" s="32">
         <v>-12.33</v>
       </c>
-      <c r="L21" s="32"/>
+      <c r="L21" s="33"/>
     </row>
     <row r="22" ht="15.0" customHeight="1">
-      <c r="A22" s="29" t="s">
-        <v>215</v>
-      </c>
-      <c r="B22" s="30">
+      <c r="A22" s="30" t="s">
+        <v>216</v>
+      </c>
+      <c r="B22" s="31">
         <v>1398.39</v>
       </c>
-      <c r="C22" s="30">
+      <c r="C22" s="31">
         <v>1119.79</v>
       </c>
-      <c r="D22" s="30">
+      <c r="D22" s="31">
         <v>794.64</v>
       </c>
-      <c r="E22" s="30">
+      <c r="E22" s="31">
         <v>583.71</v>
       </c>
-      <c r="F22" s="30">
+      <c r="F22" s="31">
         <v>354.4</v>
       </c>
-      <c r="G22" s="30">
+      <c r="G22" s="31">
         <v>213.68</v>
       </c>
-      <c r="H22" s="32"/>
-      <c r="I22" s="32"/>
-      <c r="J22" s="32"/>
-      <c r="K22" s="32"/>
-      <c r="L22" s="32"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
     </row>
     <row r="23" ht="15.0" customHeight="1">
-      <c r="A23" s="27" t="s">
-        <v>216</v>
-      </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="28"/>
-      <c r="K23" s="28"/>
-      <c r="L23" s="28"/>
+      <c r="A23" s="28" t="s">
+        <v>217</v>
+      </c>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="29"/>
     </row>
     <row r="24" ht="15.0" customHeight="1">
-      <c r="A24" s="29" t="s">
-        <v>216</v>
-      </c>
-      <c r="B24" s="30">
+      <c r="A24" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="B24" s="31">
         <v>666.22</v>
       </c>
-      <c r="C24" s="30">
+      <c r="C24" s="31">
         <v>572.63</v>
       </c>
-      <c r="D24" s="30">
+      <c r="D24" s="31">
         <v>477.06</v>
       </c>
-      <c r="E24" s="30">
+      <c r="E24" s="31">
         <v>775.0</v>
       </c>
-      <c r="F24" s="30">
+      <c r="F24" s="31">
         <v>136.97</v>
       </c>
-      <c r="G24" s="30">
+      <c r="G24" s="31">
         <v>104.89</v>
       </c>
-      <c r="H24" s="33">
+      <c r="H24" s="34">
         <v>63.29</v>
       </c>
-      <c r="I24" s="33">
+      <c r="I24" s="34">
         <v>69.53</v>
       </c>
-      <c r="J24" s="33">
+      <c r="J24" s="34">
         <v>69.56</v>
       </c>
-      <c r="K24" s="33">
+      <c r="K24" s="34">
         <v>15.85</v>
       </c>
-      <c r="L24" s="32"/>
+      <c r="L24" s="33"/>
     </row>
     <row r="25" ht="15.0" customHeight="1">
-      <c r="A25" s="29" t="s">
-        <v>217</v>
-      </c>
-      <c r="B25" s="30">
+      <c r="A25" s="30" t="s">
+        <v>218</v>
+      </c>
+      <c r="B25" s="31">
         <v>544.94</v>
       </c>
-      <c r="C25" s="30">
+      <c r="C25" s="31">
         <v>425.68</v>
       </c>
-      <c r="D25" s="30">
+      <c r="D25" s="31">
         <v>303.12</v>
       </c>
-      <c r="E25" s="30">
+      <c r="E25" s="31">
         <v>228.53</v>
       </c>
-      <c r="F25" s="33">
+      <c r="F25" s="34">
         <v>94.13</v>
       </c>
-      <c r="G25" s="33">
+      <c r="G25" s="34">
         <v>62.77</v>
       </c>
-      <c r="H25" s="32"/>
-      <c r="I25" s="32"/>
-      <c r="J25" s="32"/>
-      <c r="K25" s="32"/>
-      <c r="L25" s="32"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="33"/>
+      <c r="J25" s="33"/>
+      <c r="K25" s="33"/>
+      <c r="L25" s="33"/>
     </row>
     <row r="26" ht="15.0" customHeight="1">
-      <c r="A26" s="27" t="s">
-        <v>218</v>
-      </c>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="28"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="28"/>
-      <c r="K26" s="28"/>
-      <c r="L26" s="28"/>
+      <c r="A26" s="28" t="s">
+        <v>219</v>
+      </c>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="29"/>
+      <c r="I26" s="29"/>
+      <c r="J26" s="29"/>
+      <c r="K26" s="29"/>
+      <c r="L26" s="29"/>
     </row>
     <row r="27" ht="15.0" customHeight="1">
-      <c r="A27" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="B27" s="33">
+      <c r="A27" s="30" t="s">
+        <v>220</v>
+      </c>
+      <c r="B27" s="34">
         <v>10.28</v>
       </c>
-      <c r="C27" s="33">
+      <c r="C27" s="34">
         <v>8.46</v>
       </c>
-      <c r="D27" s="33">
+      <c r="D27" s="34">
         <v>7.31</v>
       </c>
-      <c r="E27" s="33">
+      <c r="E27" s="34">
         <v>12.28</v>
       </c>
-      <c r="F27" s="33">
+      <c r="F27" s="34">
         <v>6.63</v>
       </c>
-      <c r="G27" s="33">
+      <c r="G27" s="34">
         <v>7.08</v>
       </c>
-      <c r="H27" s="33">
+      <c r="H27" s="34">
         <v>4.51</v>
       </c>
-      <c r="I27" s="33">
+      <c r="I27" s="34">
         <v>5.06</v>
       </c>
-      <c r="J27" s="33">
+      <c r="J27" s="34">
         <v>5.2</v>
       </c>
-      <c r="K27" s="33">
+      <c r="K27" s="34">
         <v>4.27</v>
       </c>
-      <c r="L27" s="32"/>
+      <c r="L27" s="33"/>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="29" t="s">
-        <v>220</v>
-      </c>
-      <c r="B28" s="33">
+      <c r="A28" s="30" t="s">
+        <v>221</v>
+      </c>
+      <c r="B28" s="34">
         <v>9.28</v>
       </c>
-      <c r="C28" s="33">
+      <c r="C28" s="34">
         <v>8.59</v>
       </c>
-      <c r="D28" s="33">
+      <c r="D28" s="34">
         <v>7.32</v>
       </c>
-      <c r="E28" s="33">
+      <c r="E28" s="34">
         <v>7.05</v>
       </c>
-      <c r="F28" s="33">
+      <c r="F28" s="34">
         <v>6.07</v>
       </c>
-      <c r="G28" s="33">
+      <c r="G28" s="34">
         <v>5.02</v>
       </c>
-      <c r="H28" s="32"/>
-      <c r="I28" s="32"/>
-      <c r="J28" s="32"/>
-      <c r="K28" s="32"/>
-      <c r="L28" s="32"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="33"/>
+      <c r="K28" s="33"/>
+      <c r="L28" s="33"/>
     </row>
     <row r="29" ht="15.0" customHeight="1">
-      <c r="A29" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="28"/>
+      <c r="A29" s="28" t="s">
+        <v>222</v>
+      </c>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="29"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="29"/>
+      <c r="K29" s="29"/>
+      <c r="L29" s="29"/>
     </row>
     <row r="30" ht="15.0" customHeight="1">
-      <c r="A30" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="B30" s="34">
+      <c r="A30" s="30" t="s">
+        <v>223</v>
+      </c>
+      <c r="B30" s="35">
         <v>-7.19</v>
       </c>
-      <c r="C30" s="34">
+      <c r="C30" s="35">
         <v>-13.78</v>
       </c>
-      <c r="D30" s="34">
+      <c r="D30" s="35">
         <v>-19.83</v>
       </c>
-      <c r="E30" s="34">
+      <c r="E30" s="35">
         <v>-99.73</v>
       </c>
-      <c r="F30" s="34">
+      <c r="F30" s="35">
         <v>-139.36</v>
       </c>
-      <c r="G30" s="34">
+      <c r="G30" s="35">
         <v>-175.87</v>
       </c>
-      <c r="H30" s="34">
+      <c r="H30" s="35">
         <v>-24.38</v>
       </c>
-      <c r="I30" s="34">
+      <c r="I30" s="35">
         <v>-34.04</v>
       </c>
-      <c r="J30" s="34">
+      <c r="J30" s="35">
         <v>-97.86</v>
       </c>
-      <c r="K30" s="34">
+      <c r="K30" s="35">
         <v>-214.17</v>
       </c>
-      <c r="L30" s="35"/>
+      <c r="L30" s="36"/>
     </row>
     <row r="31" ht="15.0" customHeight="1">
-      <c r="A31" s="29" t="s">
-        <v>223</v>
-      </c>
-      <c r="B31" s="34">
+      <c r="A31" s="30" t="s">
+        <v>224</v>
+      </c>
+      <c r="B31" s="35">
         <v>-55.04</v>
       </c>
-      <c r="C31" s="34">
+      <c r="C31" s="35">
         <v>-87.63</v>
       </c>
-      <c r="D31" s="34">
+      <c r="D31" s="35">
         <v>-96.06</v>
       </c>
-      <c r="E31" s="34">
+      <c r="E31" s="35">
         <v>-103.77</v>
       </c>
-      <c r="F31" s="34">
+      <c r="F31" s="35">
         <v>-104.41</v>
       </c>
-      <c r="G31" s="34">
+      <c r="G31" s="35">
         <v>-112.86</v>
       </c>
-      <c r="H31" s="35"/>
-      <c r="I31" s="35"/>
-      <c r="J31" s="35"/>
-      <c r="K31" s="35"/>
-      <c r="L31" s="35"/>
+      <c r="H31" s="36"/>
+      <c r="I31" s="36"/>
+      <c r="J31" s="36"/>
+      <c r="K31" s="36"/>
+      <c r="L31" s="36"/>
     </row>
     <row r="32" ht="15.0" customHeight="1">
-      <c r="A32" s="27" t="s">
-        <v>224</v>
-      </c>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
+      <c r="A32" s="28" t="s">
+        <v>225</v>
+      </c>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="29"/>
+      <c r="J32" s="29"/>
+      <c r="K32" s="29"/>
+      <c r="L32" s="29"/>
     </row>
     <row r="33" ht="15.0" customHeight="1">
-      <c r="A33" s="29" t="s">
-        <v>225</v>
-      </c>
-      <c r="B33" s="35">
+      <c r="A33" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="B33" s="36">
         <v>2.1</v>
       </c>
-      <c r="C33" s="35">
+      <c r="C33" s="36">
         <v>3.33</v>
       </c>
-      <c r="D33" s="35">
+      <c r="D33" s="36">
         <v>1.8</v>
       </c>
-      <c r="E33" s="35">
+      <c r="E33" s="36">
         <v>3.33</v>
       </c>
-      <c r="F33" s="35">
+      <c r="F33" s="36">
         <v>4.41</v>
       </c>
-      <c r="G33" s="35">
+      <c r="G33" s="36">
         <v>0.0</v>
       </c>
-      <c r="H33" s="35">
+      <c r="H33" s="36">
         <v>0.0</v>
       </c>
-      <c r="I33" s="35">
+      <c r="I33" s="36">
         <v>0.0</v>
       </c>
-      <c r="J33" s="35">
+      <c r="J33" s="36">
         <v>0.0</v>
       </c>
-      <c r="K33" s="35">
+      <c r="K33" s="36">
         <v>0.0</v>
       </c>
-      <c r="L33" s="35"/>
+      <c r="L33" s="36"/>
     </row>
     <row r="34" ht="15.0" customHeight="1">
-      <c r="A34" s="29" t="s">
-        <v>226</v>
-      </c>
-      <c r="B34" s="35">
+      <c r="A34" s="30" t="s">
+        <v>227</v>
+      </c>
+      <c r="B34" s="36">
         <v>2.95</v>
       </c>
-      <c r="C34" s="35">
+      <c r="C34" s="36">
         <v>2.62</v>
       </c>
-      <c r="D34" s="35">
+      <c r="D34" s="36">
         <v>2.16</v>
       </c>
-      <c r="E34" s="35">
+      <c r="E34" s="36">
         <v>1.94</v>
       </c>
-      <c r="F34" s="35">
+      <c r="F34" s="36">
         <v>0.96</v>
       </c>
-      <c r="G34" s="35">
+      <c r="G34" s="36">
         <v>0.0</v>
       </c>
-      <c r="H34" s="35"/>
-      <c r="I34" s="35"/>
-      <c r="J34" s="35"/>
-      <c r="K34" s="35"/>
-      <c r="L34" s="35"/>
+      <c r="H34" s="36"/>
+      <c r="I34" s="36"/>
+      <c r="J34" s="36"/>
+      <c r="K34" s="36"/>
+      <c r="L34" s="36"/>
     </row>
     <row r="35" ht="15.0" customHeight="1">
-      <c r="A35" s="29" t="s">
-        <v>227</v>
-      </c>
-      <c r="B35" s="35">
+      <c r="A35" s="30" t="s">
+        <v>228</v>
+      </c>
+      <c r="B35" s="36">
         <v>3.0</v>
       </c>
-      <c r="C35" s="35">
+      <c r="C35" s="36">
         <v>4.76</v>
       </c>
-      <c r="D35" s="35">
+      <c r="D35" s="36">
         <v>2.57</v>
       </c>
-      <c r="E35" s="35">
+      <c r="E35" s="36">
         <v>4.76</v>
       </c>
-      <c r="F35" s="35">
+      <c r="F35" s="36">
         <v>6.3</v>
       </c>
-      <c r="G35" s="35">
+      <c r="G35" s="36">
         <v>0.0</v>
       </c>
-      <c r="H35" s="35">
+      <c r="H35" s="36">
         <v>0.0</v>
       </c>
-      <c r="I35" s="35">
+      <c r="I35" s="36">
         <v>0.0</v>
       </c>
-      <c r="J35" s="35">
+      <c r="J35" s="36">
         <v>0.0</v>
       </c>
-      <c r="K35" s="35">
+      <c r="K35" s="36">
         <v>0.0</v>
       </c>
-      <c r="L35" s="35"/>
+      <c r="L35" s="36"/>
     </row>
     <row r="36" ht="15.0" customHeight="1">
-      <c r="A36" s="29" t="s">
-        <v>228</v>
-      </c>
-      <c r="B36" s="35">
+      <c r="A36" s="30" t="s">
+        <v>229</v>
+      </c>
+      <c r="B36" s="36">
         <v>4.21</v>
       </c>
-      <c r="C36" s="35">
+      <c r="C36" s="36">
         <v>3.75</v>
       </c>
-      <c r="D36" s="35">
+      <c r="D36" s="36">
         <v>3.09</v>
       </c>
-      <c r="E36" s="35">
+      <c r="E36" s="36">
         <v>2.76</v>
       </c>
-      <c r="F36" s="35">
+      <c r="F36" s="36">
         <v>1.38</v>
       </c>
-      <c r="G36" s="35">
+      <c r="G36" s="36">
         <v>0.0</v>
       </c>
-      <c r="H36" s="35"/>
-      <c r="I36" s="35"/>
-      <c r="J36" s="35"/>
-      <c r="K36" s="35"/>
-      <c r="L36" s="35"/>
+      <c r="H36" s="36"/>
+      <c r="I36" s="36"/>
+      <c r="J36" s="36"/>
+      <c r="K36" s="36"/>
+      <c r="L36" s="36"/>
     </row>
     <row r="37" ht="15.0" customHeight="1">
-      <c r="A37" s="27" t="s">
-        <v>229</v>
-      </c>
-      <c r="B37" s="28"/>
-      <c r="C37" s="28"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="28"/>
-      <c r="F37" s="28"/>
-      <c r="G37" s="28"/>
-      <c r="H37" s="28"/>
-      <c r="I37" s="28"/>
-      <c r="J37" s="28"/>
-      <c r="K37" s="28"/>
-      <c r="L37" s="28"/>
+      <c r="A37" s="28" t="s">
+        <v>230</v>
+      </c>
+      <c r="B37" s="29"/>
+      <c r="C37" s="29"/>
+      <c r="D37" s="29"/>
+      <c r="E37" s="29"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="29"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="29"/>
+      <c r="J37" s="29"/>
+      <c r="K37" s="29"/>
+      <c r="L37" s="29"/>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="29" t="s">
-        <v>230</v>
-      </c>
-      <c r="B38" s="33">
+      <c r="A38" s="30" t="s">
+        <v>231</v>
+      </c>
+      <c r="B38" s="34">
         <v>0.71</v>
       </c>
-      <c r="C38" s="33">
+      <c r="C38" s="34">
         <v>0.61</v>
       </c>
-      <c r="D38" s="33">
+      <c r="D38" s="34">
         <v>0.53</v>
       </c>
-      <c r="E38" s="33">
+      <c r="E38" s="34">
         <v>0.93</v>
       </c>
-      <c r="F38" s="33">
+      <c r="F38" s="34">
         <v>0.28</v>
       </c>
-      <c r="G38" s="33">
+      <c r="G38" s="34">
         <v>0.35</v>
       </c>
-      <c r="H38" s="33">
+      <c r="H38" s="34">
         <v>0.74</v>
       </c>
-      <c r="I38" s="33">
+      <c r="I38" s="34">
         <v>0.89</v>
       </c>
-      <c r="J38" s="33">
+      <c r="J38" s="34">
         <v>1.2</v>
       </c>
-      <c r="K38" s="33">
+      <c r="K38" s="34">
         <v>0.36</v>
       </c>
-      <c r="L38" s="32"/>
+      <c r="L38" s="33"/>
     </row>
     <row r="39" ht="15.0" customHeight="1">
-      <c r="A39" s="29" t="s">
-        <v>231</v>
-      </c>
-      <c r="B39" s="33">
+      <c r="A39" s="30" t="s">
+        <v>232</v>
+      </c>
+      <c r="B39" s="34">
         <v>0.57</v>
       </c>
-      <c r="C39" s="33">
+      <c r="C39" s="34">
         <v>0.49</v>
       </c>
-      <c r="D39" s="33">
+      <c r="D39" s="34">
         <v>0.49</v>
       </c>
-      <c r="E39" s="33">
+      <c r="E39" s="34">
         <v>0.52</v>
       </c>
-      <c r="F39" s="33">
+      <c r="F39" s="34">
         <v>0.48</v>
       </c>
-      <c r="G39" s="33">
+      <c r="G39" s="34">
         <v>0.54</v>
       </c>
-      <c r="H39" s="32"/>
-      <c r="I39" s="32"/>
-      <c r="J39" s="32"/>
-      <c r="K39" s="32"/>
-      <c r="L39" s="32"/>
+      <c r="H39" s="33"/>
+      <c r="I39" s="33"/>
+      <c r="J39" s="33"/>
+      <c r="K39" s="33"/>
+      <c r="L39" s="33"/>
     </row>
     <row r="40" ht="15.0" customHeight="1">
-      <c r="A40" s="27" t="s">
-        <v>232</v>
-      </c>
-      <c r="B40" s="28"/>
-      <c r="C40" s="28"/>
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="28"/>
-      <c r="H40" s="28"/>
-      <c r="I40" s="28"/>
-      <c r="J40" s="28"/>
-      <c r="K40" s="28"/>
-      <c r="L40" s="28"/>
+      <c r="A40" s="28" t="s">
+        <v>233</v>
+      </c>
+      <c r="B40" s="29"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="29"/>
+      <c r="I40" s="29"/>
+      <c r="J40" s="29"/>
+      <c r="K40" s="29"/>
+      <c r="L40" s="29"/>
     </row>
     <row r="41" ht="15.0" customHeight="1">
-      <c r="A41" s="29" t="s">
-        <v>233</v>
-      </c>
-      <c r="B41" s="33">
+      <c r="A41" s="30" t="s">
+        <v>234</v>
+      </c>
+      <c r="B41" s="34">
         <v>0.74</v>
       </c>
-      <c r="C41" s="33">
+      <c r="C41" s="34">
         <v>0.63</v>
       </c>
-      <c r="D41" s="33">
+      <c r="D41" s="34">
         <v>0.56</v>
       </c>
-      <c r="E41" s="33">
+      <c r="E41" s="34">
         <v>0.98</v>
       </c>
-      <c r="F41" s="33">
+      <c r="F41" s="34">
         <v>0.31</v>
       </c>
-      <c r="G41" s="33">
+      <c r="G41" s="34">
         <v>0.4</v>
       </c>
-      <c r="H41" s="33">
+      <c r="H41" s="34">
         <v>0.91</v>
       </c>
-      <c r="I41" s="33">
+      <c r="I41" s="34">
         <v>1.13</v>
       </c>
-      <c r="J41" s="33">
+      <c r="J41" s="34">
         <v>1.57</v>
       </c>
-      <c r="K41" s="33">
+      <c r="K41" s="34">
         <v>0.36</v>
       </c>
-      <c r="L41" s="32"/>
+      <c r="L41" s="33"/>
     </row>
     <row r="42" ht="15.0" customHeight="1">
-      <c r="A42" s="29" t="s">
-        <v>234</v>
-      </c>
-      <c r="B42" s="33">
+      <c r="A42" s="30" t="s">
+        <v>235</v>
+      </c>
+      <c r="B42" s="34">
         <v>0.61</v>
       </c>
-      <c r="C42" s="33">
+      <c r="C42" s="34">
         <v>0.54</v>
       </c>
-      <c r="D42" s="33">
+      <c r="D42" s="34">
         <v>0.54</v>
       </c>
-      <c r="E42" s="33">
+      <c r="E42" s="34">
         <v>0.58</v>
       </c>
-      <c r="F42" s="33">
+      <c r="F42" s="34">
         <v>0.55</v>
       </c>
-      <c r="G42" s="33">
+      <c r="G42" s="34">
         <v>0.62</v>
       </c>
-      <c r="H42" s="32"/>
-      <c r="I42" s="32"/>
-      <c r="J42" s="32"/>
-      <c r="K42" s="32"/>
-      <c r="L42" s="32"/>
+      <c r="H42" s="33"/>
+      <c r="I42" s="33"/>
+      <c r="J42" s="33"/>
+      <c r="K42" s="33"/>
+      <c r="L42" s="33"/>
     </row>
     <row r="43" ht="15.0" customHeight="1">
-      <c r="A43" s="27" t="s">
-        <v>235</v>
-      </c>
-      <c r="B43" s="28"/>
-      <c r="C43" s="28"/>
-      <c r="D43" s="28"/>
-      <c r="E43" s="28"/>
-      <c r="F43" s="28"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="28"/>
-      <c r="I43" s="28"/>
-      <c r="J43" s="28"/>
-      <c r="K43" s="28"/>
-      <c r="L43" s="28"/>
+      <c r="A43" s="28" t="s">
+        <v>236</v>
+      </c>
+      <c r="B43" s="29"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="29"/>
+      <c r="I43" s="29"/>
+      <c r="J43" s="29"/>
+      <c r="K43" s="29"/>
+      <c r="L43" s="29"/>
     </row>
     <row r="44" ht="15.0" customHeight="1">
-      <c r="A44" s="29" t="s">
-        <v>236</v>
-      </c>
-      <c r="B44" s="33">
+      <c r="A44" s="30" t="s">
+        <v>237</v>
+      </c>
+      <c r="B44" s="34">
         <v>4.29</v>
       </c>
-      <c r="C44" s="33">
+      <c r="C44" s="34">
         <v>3.86</v>
       </c>
-      <c r="D44" s="33">
+      <c r="D44" s="34">
         <v>3.85</v>
       </c>
-      <c r="E44" s="33">
+      <c r="E44" s="34">
         <v>5.28</v>
       </c>
-      <c r="F44" s="33">
+      <c r="F44" s="34">
         <v>1.14</v>
       </c>
-      <c r="G44" s="33">
+      <c r="G44" s="34">
         <v>1.31</v>
       </c>
-      <c r="H44" s="33">
+      <c r="H44" s="34">
         <v>2.22</v>
       </c>
-      <c r="I44" s="33">
+      <c r="I44" s="34">
         <v>2.49</v>
       </c>
-      <c r="J44" s="33">
+      <c r="J44" s="34">
         <v>6.97</v>
       </c>
-      <c r="K44" s="33">
+      <c r="K44" s="34">
         <v>2.88</v>
       </c>
-      <c r="L44" s="32"/>
+      <c r="L44" s="33"/>
     </row>
     <row r="45" ht="15.0" customHeight="1">
-      <c r="A45" s="29" t="s">
-        <v>237</v>
-      </c>
-      <c r="B45" s="33">
+      <c r="A45" s="30" t="s">
+        <v>238</v>
+      </c>
+      <c r="B45" s="34">
         <v>3.12</v>
       </c>
-      <c r="C45" s="33">
+      <c r="C45" s="34">
         <v>2.38</v>
       </c>
-      <c r="D45" s="33">
+      <c r="D45" s="34">
         <v>2.18</v>
       </c>
-      <c r="E45" s="33">
+      <c r="E45" s="34">
         <v>2.03</v>
       </c>
-      <c r="F45" s="33">
+      <c r="F45" s="34">
         <v>1.79</v>
       </c>
-      <c r="G45" s="33">
+      <c r="G45" s="34">
         <v>2.22</v>
       </c>
-      <c r="H45" s="32"/>
-      <c r="I45" s="32"/>
-      <c r="J45" s="32"/>
-      <c r="K45" s="32"/>
-      <c r="L45" s="32"/>
+      <c r="H45" s="33"/>
+      <c r="I45" s="33"/>
+      <c r="J45" s="33"/>
+      <c r="K45" s="33"/>
+      <c r="L45" s="33"/>
     </row>
     <row r="46" ht="15.0" customHeight="1">
-      <c r="A46" s="27" t="s">
-        <v>238</v>
-      </c>
-      <c r="B46" s="28"/>
-      <c r="C46" s="28"/>
-      <c r="D46" s="28"/>
-      <c r="E46" s="28"/>
-      <c r="F46" s="28"/>
-      <c r="G46" s="28"/>
-      <c r="H46" s="28"/>
-      <c r="I46" s="28"/>
-      <c r="J46" s="28"/>
-      <c r="K46" s="28"/>
-      <c r="L46" s="28"/>
+      <c r="A46" s="28" t="s">
+        <v>239</v>
+      </c>
+      <c r="B46" s="29"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
+      <c r="H46" s="29"/>
+      <c r="I46" s="29"/>
+      <c r="J46" s="29"/>
+      <c r="K46" s="29"/>
+      <c r="L46" s="29"/>
     </row>
     <row r="47" ht="15.0" customHeight="1">
-      <c r="A47" s="29" t="s">
-        <v>239</v>
-      </c>
-      <c r="B47" s="33">
+      <c r="A47" s="30" t="s">
+        <v>240</v>
+      </c>
+      <c r="B47" s="34">
         <v>18.4</v>
       </c>
-      <c r="C47" s="33">
+      <c r="C47" s="34">
         <v>58.37</v>
       </c>
-      <c r="D47" s="33">
+      <c r="D47" s="34">
         <v>5.98</v>
       </c>
-      <c r="E47" s="33">
+      <c r="E47" s="34">
         <v>3.46</v>
       </c>
-      <c r="F47" s="33">
+      <c r="F47" s="34">
         <v>2.86</v>
       </c>
-      <c r="G47" s="33">
+      <c r="G47" s="34">
         <v>2.98</v>
       </c>
-      <c r="H47" s="33">
+      <c r="H47" s="34">
         <v>5.75</v>
       </c>
-      <c r="I47" s="33">
+      <c r="I47" s="34">
         <v>4.51</v>
       </c>
-      <c r="J47" s="33">
+      <c r="J47" s="34">
         <v>11.71</v>
       </c>
-      <c r="K47" s="32"/>
-      <c r="L47" s="32"/>
+      <c r="K47" s="33"/>
+      <c r="L47" s="33"/>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="29" t="s">
-        <v>240</v>
-      </c>
-      <c r="B48" s="33">
+      <c r="A48" s="30" t="s">
+        <v>241</v>
+      </c>
+      <c r="B48" s="34">
         <v>5.75</v>
       </c>
-      <c r="C48" s="33">
+      <c r="C48" s="34">
         <v>4.34</v>
       </c>
-      <c r="D48" s="33">
+      <c r="D48" s="34">
         <v>3.7</v>
       </c>
-      <c r="E48" s="33">
+      <c r="E48" s="34">
         <v>3.5</v>
       </c>
-      <c r="F48" s="33">
+      <c r="F48" s="34">
         <v>4.07</v>
       </c>
-      <c r="G48" s="32"/>
-      <c r="H48" s="32"/>
-      <c r="I48" s="32"/>
-      <c r="J48" s="32"/>
-      <c r="K48" s="32"/>
-      <c r="L48" s="32"/>
+      <c r="G48" s="33"/>
+      <c r="H48" s="33"/>
+      <c r="I48" s="33"/>
+      <c r="J48" s="33"/>
+      <c r="K48" s="33"/>
+      <c r="L48" s="33"/>
     </row>
     <row r="49" ht="15.0" customHeight="1">
-      <c r="A49" s="27" t="s">
-        <v>241</v>
-      </c>
-      <c r="B49" s="28"/>
-      <c r="C49" s="28"/>
-      <c r="D49" s="28"/>
-      <c r="E49" s="28"/>
-      <c r="F49" s="28"/>
-      <c r="G49" s="28"/>
-      <c r="H49" s="28"/>
-      <c r="I49" s="28"/>
-      <c r="J49" s="28"/>
-      <c r="K49" s="28"/>
-      <c r="L49" s="28"/>
+      <c r="A49" s="28" t="s">
+        <v>242</v>
+      </c>
+      <c r="B49" s="29"/>
+      <c r="C49" s="29"/>
+      <c r="D49" s="29"/>
+      <c r="E49" s="29"/>
+      <c r="F49" s="29"/>
+      <c r="G49" s="29"/>
+      <c r="H49" s="29"/>
+      <c r="I49" s="29"/>
+      <c r="J49" s="29"/>
+      <c r="K49" s="29"/>
+      <c r="L49" s="29"/>
     </row>
     <row r="50" ht="15.0" customHeight="1">
-      <c r="A50" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="B50" s="33">
+      <c r="A50" s="30" t="s">
+        <v>243</v>
+      </c>
+      <c r="B50" s="34">
         <v>19.09</v>
       </c>
-      <c r="C50" s="33">
+      <c r="C50" s="34">
         <v>73.2</v>
       </c>
-      <c r="D50" s="33">
+      <c r="D50" s="34">
         <v>6.34</v>
       </c>
-      <c r="E50" s="33">
+      <c r="E50" s="34">
         <v>3.51</v>
       </c>
-      <c r="F50" s="33">
+      <c r="F50" s="34">
         <v>2.92</v>
       </c>
-      <c r="G50" s="33">
+      <c r="G50" s="34">
         <v>3.0</v>
       </c>
-      <c r="H50" s="33">
+      <c r="H50" s="34">
         <v>5.8</v>
       </c>
-      <c r="I50" s="33">
+      <c r="I50" s="34">
         <v>4.58</v>
       </c>
-      <c r="J50" s="33">
+      <c r="J50" s="34">
         <v>11.85</v>
       </c>
-      <c r="K50" s="33">
+      <c r="K50" s="34">
         <v>0.59</v>
       </c>
-      <c r="L50" s="32"/>
+      <c r="L50" s="33"/>
     </row>
     <row r="51" ht="15.0" customHeight="1">
-      <c r="A51" s="29" t="s">
-        <v>243</v>
-      </c>
-      <c r="B51" s="33">
+      <c r="A51" s="30" t="s">
+        <v>244</v>
+      </c>
+      <c r="B51" s="34">
         <v>5.92</v>
       </c>
-      <c r="C51" s="33">
+      <c r="C51" s="34">
         <v>4.44</v>
       </c>
-      <c r="D51" s="33">
+      <c r="D51" s="34">
         <v>3.78</v>
       </c>
-      <c r="E51" s="33">
+      <c r="E51" s="34">
         <v>3.56</v>
       </c>
-      <c r="F51" s="33">
+      <c r="F51" s="34">
         <v>4.12</v>
       </c>
-      <c r="G51" s="33">
+      <c r="G51" s="34">
         <v>2.26</v>
       </c>
-      <c r="H51" s="32"/>
-      <c r="I51" s="32"/>
-      <c r="J51" s="32"/>
-      <c r="K51" s="32"/>
-      <c r="L51" s="32"/>
+      <c r="H51" s="33"/>
+      <c r="I51" s="33"/>
+      <c r="J51" s="33"/>
+      <c r="K51" s="33"/>
+      <c r="L51" s="33"/>
     </row>
     <row r="52" ht="15.0" customHeight="1">
-      <c r="A52" s="27" t="s">
-        <v>244</v>
-      </c>
-      <c r="B52" s="28"/>
-      <c r="C52" s="28"/>
-      <c r="D52" s="28"/>
-      <c r="E52" s="28"/>
-      <c r="F52" s="28"/>
-      <c r="G52" s="28"/>
-      <c r="H52" s="28"/>
-      <c r="I52" s="28"/>
-      <c r="J52" s="28"/>
-      <c r="K52" s="28"/>
-      <c r="L52" s="28"/>
+      <c r="A52" s="28" t="s">
+        <v>245</v>
+      </c>
+      <c r="B52" s="29"/>
+      <c r="C52" s="29"/>
+      <c r="D52" s="29"/>
+      <c r="E52" s="29"/>
+      <c r="F52" s="29"/>
+      <c r="G52" s="29"/>
+      <c r="H52" s="29"/>
+      <c r="I52" s="29"/>
+      <c r="J52" s="29"/>
+      <c r="K52" s="29"/>
+      <c r="L52" s="29"/>
     </row>
     <row r="53" ht="15.0" customHeight="1">
-      <c r="A53" s="29" t="s">
-        <v>245</v>
-      </c>
-      <c r="B53" s="33">
+      <c r="A53" s="30" t="s">
+        <v>246</v>
+      </c>
+      <c r="B53" s="34">
         <v>65.28</v>
       </c>
-      <c r="C53" s="33">
+      <c r="C53" s="34">
         <v>9.94</v>
       </c>
-      <c r="D53" s="30">
+      <c r="D53" s="31">
         <v>169.93</v>
       </c>
-      <c r="E53" s="32"/>
-      <c r="F53" s="33">
+      <c r="E53" s="33"/>
+      <c r="F53" s="34">
         <v>26.04</v>
       </c>
-      <c r="G53" s="33">
+      <c r="G53" s="34">
         <v>29.81</v>
       </c>
-      <c r="H53" s="33">
+      <c r="H53" s="34">
         <v>18.76</v>
       </c>
-      <c r="I53" s="33">
+      <c r="I53" s="34">
         <v>35.03</v>
       </c>
-      <c r="J53" s="30">
+      <c r="J53" s="31">
         <v>136.17</v>
       </c>
-      <c r="K53" s="33">
+      <c r="K53" s="34">
         <v>7.56</v>
       </c>
-      <c r="L53" s="32"/>
+      <c r="L53" s="33"/>
     </row>
     <row r="54" ht="15.0" customHeight="1">
-      <c r="A54" s="29" t="s">
-        <v>246</v>
-      </c>
-      <c r="B54" s="33">
+      <c r="A54" s="30" t="s">
+        <v>247</v>
+      </c>
+      <c r="B54" s="34">
         <v>0.57</v>
       </c>
-      <c r="C54" s="33">
+      <c r="C54" s="34">
         <v>0.49</v>
       </c>
-      <c r="D54" s="33">
+      <c r="D54" s="34">
         <v>0.49</v>
       </c>
-      <c r="E54" s="33">
+      <c r="E54" s="34">
         <v>0.52</v>
       </c>
-      <c r="F54" s="33">
+      <c r="F54" s="34">
         <v>0.48</v>
       </c>
-      <c r="G54" s="33">
+      <c r="G54" s="34">
         <v>0.54</v>
       </c>
-      <c r="H54" s="32"/>
-      <c r="I54" s="32"/>
-      <c r="J54" s="32"/>
-      <c r="K54" s="32"/>
-      <c r="L54" s="32"/>
+      <c r="H54" s="33"/>
+      <c r="I54" s="33"/>
+      <c r="J54" s="33"/>
+      <c r="K54" s="33"/>
+      <c r="L54" s="33"/>
     </row>
     <row r="55" ht="15.0" customHeight="1">
-      <c r="A55" s="27" t="s">
-        <v>247</v>
-      </c>
-      <c r="B55" s="28"/>
-      <c r="C55" s="28"/>
-      <c r="D55" s="28"/>
-      <c r="E55" s="28"/>
-      <c r="F55" s="28"/>
-      <c r="G55" s="28"/>
-      <c r="H55" s="28"/>
-      <c r="I55" s="28"/>
-      <c r="J55" s="28"/>
-      <c r="K55" s="28"/>
-      <c r="L55" s="28"/>
+      <c r="A55" s="28" t="s">
+        <v>248</v>
+      </c>
+      <c r="B55" s="29"/>
+      <c r="C55" s="29"/>
+      <c r="D55" s="29"/>
+      <c r="E55" s="29"/>
+      <c r="F55" s="29"/>
+      <c r="G55" s="29"/>
+      <c r="H55" s="29"/>
+      <c r="I55" s="29"/>
+      <c r="J55" s="29"/>
+      <c r="K55" s="29"/>
+      <c r="L55" s="29"/>
     </row>
     <row r="56" ht="15.0" customHeight="1">
-      <c r="A56" s="29" t="s">
-        <v>248</v>
-      </c>
-      <c r="B56" s="33">
+      <c r="A56" s="30" t="s">
+        <v>249</v>
+      </c>
+      <c r="B56" s="34">
         <v>0.05</v>
       </c>
-      <c r="C56" s="31">
+      <c r="C56" s="32">
         <v>-0.81</v>
       </c>
-      <c r="D56" s="31">
+      <c r="D56" s="32">
         <v>-0.1</v>
       </c>
-      <c r="E56" s="33">
+      <c r="E56" s="34">
         <v>0.05</v>
       </c>
-      <c r="F56" s="31">
+      <c r="F56" s="32">
         <v>-0.22</v>
       </c>
-      <c r="G56" s="33">
+      <c r="G56" s="34">
         <v>0.01</v>
       </c>
-      <c r="H56" s="31">
+      <c r="H56" s="32">
         <v>-0.21</v>
       </c>
-      <c r="I56" s="33">
+      <c r="I56" s="34">
         <v>0.03</v>
       </c>
-      <c r="J56" s="31">
+      <c r="J56" s="32">
         <v>-0.13</v>
       </c>
-      <c r="K56" s="32"/>
-      <c r="L56" s="32"/>
+      <c r="K56" s="33"/>
+      <c r="L56" s="33"/>
     </row>
     <row r="57" ht="15.0" customHeight="1">
-      <c r="A57" s="29" t="s">
-        <v>249</v>
-      </c>
-      <c r="B57" s="31">
+      <c r="A57" s="30" t="s">
+        <v>250</v>
+      </c>
+      <c r="B57" s="32">
         <v>-0.22</v>
       </c>
-      <c r="C57" s="31">
+      <c r="C57" s="32">
         <v>-0.14</v>
       </c>
-      <c r="D57" s="33">
+      <c r="D57" s="34">
         <v>1.78</v>
       </c>
-      <c r="E57" s="33">
+      <c r="E57" s="34">
         <v>0.07</v>
       </c>
-      <c r="F57" s="31">
+      <c r="F57" s="32">
         <v>-0.2</v>
       </c>
-      <c r="G57" s="32"/>
-      <c r="H57" s="32"/>
-      <c r="I57" s="32"/>
-      <c r="J57" s="32"/>
-      <c r="K57" s="32"/>
-      <c r="L57" s="32"/>
+      <c r="G57" s="33"/>
+      <c r="H57" s="33"/>
+      <c r="I57" s="33"/>
+      <c r="J57" s="33"/>
+      <c r="K57" s="33"/>
+      <c r="L57" s="33"/>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="27" t="s">
-        <v>250</v>
-      </c>
-      <c r="B58" s="28"/>
-      <c r="C58" s="28"/>
-      <c r="D58" s="28"/>
-      <c r="E58" s="28"/>
-      <c r="F58" s="28"/>
-      <c r="G58" s="28"/>
-      <c r="H58" s="28"/>
-      <c r="I58" s="28"/>
-      <c r="J58" s="28"/>
-      <c r="K58" s="28"/>
-      <c r="L58" s="28"/>
+      <c r="A58" s="28" t="s">
+        <v>251</v>
+      </c>
+      <c r="B58" s="29"/>
+      <c r="C58" s="29"/>
+      <c r="D58" s="29"/>
+      <c r="E58" s="29"/>
+      <c r="F58" s="29"/>
+      <c r="G58" s="29"/>
+      <c r="H58" s="29"/>
+      <c r="I58" s="29"/>
+      <c r="J58" s="29"/>
+      <c r="K58" s="29"/>
+      <c r="L58" s="29"/>
     </row>
     <row r="59" ht="15.0" customHeight="1">
-      <c r="A59" s="29" t="s">
-        <v>251</v>
-      </c>
-      <c r="B59" s="33">
+      <c r="A59" s="30" t="s">
+        <v>252</v>
+      </c>
+      <c r="B59" s="34">
         <v>10.29</v>
       </c>
-      <c r="C59" s="33">
+      <c r="C59" s="34">
         <v>11.0</v>
       </c>
-      <c r="D59" s="33">
+      <c r="D59" s="34">
         <v>11.29</v>
       </c>
-      <c r="E59" s="33">
+      <c r="E59" s="34">
         <v>14.9</v>
       </c>
-      <c r="F59" s="33">
+      <c r="F59" s="34">
         <v>4.99</v>
       </c>
-      <c r="G59" s="33">
+      <c r="G59" s="34">
         <v>4.29</v>
       </c>
-      <c r="H59" s="33">
+      <c r="H59" s="34">
         <v>3.17</v>
       </c>
-      <c r="I59" s="33">
+      <c r="I59" s="34">
         <v>2.97</v>
       </c>
-      <c r="J59" s="33">
+      <c r="J59" s="34">
         <v>7.0</v>
       </c>
-      <c r="K59" s="31">
+      <c r="K59" s="32">
         <v>-2.24</v>
       </c>
-      <c r="L59" s="32"/>
+      <c r="L59" s="33"/>
     </row>
     <row r="60" ht="15.0" customHeight="1">
-      <c r="A60" s="29" t="s">
-        <v>252</v>
-      </c>
-      <c r="B60" s="33">
+      <c r="A60" s="30" t="s">
+        <v>253</v>
+      </c>
+      <c r="B60" s="34">
         <v>10.48</v>
       </c>
-      <c r="C60" s="33">
+      <c r="C60" s="34">
         <v>9.54</v>
       </c>
-      <c r="D60" s="33">
+      <c r="D60" s="34">
         <v>8.06</v>
       </c>
-      <c r="E60" s="33">
+      <c r="E60" s="34">
         <v>6.28</v>
       </c>
-      <c r="F60" s="33">
+      <c r="F60" s="34">
         <v>4.17</v>
       </c>
-      <c r="G60" s="33">
+      <c r="G60" s="34">
         <v>3.77</v>
       </c>
-      <c r="H60" s="32"/>
-      <c r="I60" s="32"/>
-      <c r="J60" s="32"/>
-      <c r="K60" s="32"/>
-      <c r="L60" s="32"/>
+      <c r="H60" s="33"/>
+      <c r="I60" s="33"/>
+      <c r="J60" s="33"/>
+      <c r="K60" s="33"/>
+      <c r="L60" s="33"/>
     </row>
     <row r="61" ht="15.0" customHeight="1">
-      <c r="A61" s="27" t="s">
-        <v>253</v>
-      </c>
-      <c r="B61" s="28"/>
-      <c r="C61" s="28"/>
-      <c r="D61" s="28"/>
-      <c r="E61" s="28"/>
-      <c r="F61" s="28"/>
-      <c r="G61" s="28"/>
-      <c r="H61" s="28"/>
-      <c r="I61" s="28"/>
-      <c r="J61" s="28"/>
-      <c r="K61" s="28"/>
-      <c r="L61" s="28"/>
+      <c r="A61" s="28" t="s">
+        <v>254</v>
+      </c>
+      <c r="B61" s="29"/>
+      <c r="C61" s="29"/>
+      <c r="D61" s="29"/>
+      <c r="E61" s="29"/>
+      <c r="F61" s="29"/>
+      <c r="G61" s="29"/>
+      <c r="H61" s="29"/>
+      <c r="I61" s="29"/>
+      <c r="J61" s="29"/>
+      <c r="K61" s="29"/>
+      <c r="L61" s="29"/>
     </row>
     <row r="62" ht="15.0" customHeight="1">
-      <c r="A62" s="29" t="s">
-        <v>254</v>
-      </c>
-      <c r="B62" s="33">
+      <c r="A62" s="30" t="s">
+        <v>255</v>
+      </c>
+      <c r="B62" s="34">
         <v>17.74</v>
       </c>
-      <c r="C62" s="33">
+      <c r="C62" s="34">
         <v>21.83</v>
       </c>
-      <c r="D62" s="33">
+      <c r="D62" s="34">
         <v>26.39</v>
       </c>
-      <c r="E62" s="33">
+      <c r="E62" s="34">
         <v>41.87</v>
       </c>
-      <c r="F62" s="33">
+      <c r="F62" s="34">
         <v>18.8</v>
       </c>
-      <c r="G62" s="33">
+      <c r="G62" s="34">
         <v>20.21</v>
       </c>
-      <c r="H62" s="33">
+      <c r="H62" s="34">
         <v>12.15</v>
       </c>
-      <c r="I62" s="33">
+      <c r="I62" s="34">
         <v>10.64</v>
       </c>
-      <c r="J62" s="33">
+      <c r="J62" s="34">
         <v>42.19</v>
       </c>
-      <c r="K62" s="31">
+      <c r="K62" s="32">
         <v>-3.76</v>
       </c>
-      <c r="L62" s="32"/>
+      <c r="L62" s="33"/>
     </row>
     <row r="63" ht="15.0" customHeight="1">
-      <c r="A63" s="29" t="s">
-        <v>255</v>
-      </c>
-      <c r="B63" s="33">
+      <c r="A63" s="30" t="s">
+        <v>256</v>
+      </c>
+      <c r="B63" s="34">
         <v>23.62</v>
       </c>
-      <c r="C63" s="33">
+      <c r="C63" s="34">
         <v>25.83</v>
       </c>
-      <c r="D63" s="33">
+      <c r="D63" s="34">
         <v>25.74</v>
       </c>
-      <c r="E63" s="33">
+      <c r="E63" s="34">
         <v>22.78</v>
       </c>
-      <c r="F63" s="33">
+      <c r="F63" s="34">
         <v>16.89</v>
       </c>
-      <c r="G63" s="33">
+      <c r="G63" s="34">
         <v>15.28</v>
       </c>
-      <c r="H63" s="32"/>
-      <c r="I63" s="32"/>
-      <c r="J63" s="32"/>
-      <c r="K63" s="32"/>
-      <c r="L63" s="32"/>
+      <c r="H63" s="33"/>
+      <c r="I63" s="33"/>
+      <c r="J63" s="33"/>
+      <c r="K63" s="33"/>
+      <c r="L63" s="33"/>
     </row>
     <row r="64" ht="15.0" customHeight="1">
-      <c r="A64" s="27" t="s">
-        <v>256</v>
-      </c>
-      <c r="B64" s="28"/>
-      <c r="C64" s="28"/>
-      <c r="D64" s="28"/>
-      <c r="E64" s="28"/>
-      <c r="F64" s="28"/>
-      <c r="G64" s="28"/>
-      <c r="H64" s="28"/>
-      <c r="I64" s="28"/>
-      <c r="J64" s="28"/>
-      <c r="K64" s="28"/>
-      <c r="L64" s="28"/>
+      <c r="A64" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="B64" s="29"/>
+      <c r="C64" s="29"/>
+      <c r="D64" s="29"/>
+      <c r="E64" s="29"/>
+      <c r="F64" s="29"/>
+      <c r="G64" s="29"/>
+      <c r="H64" s="29"/>
+      <c r="I64" s="29"/>
+      <c r="J64" s="29"/>
+      <c r="K64" s="29"/>
+      <c r="L64" s="29"/>
     </row>
     <row r="65" ht="15.0" customHeight="1">
-      <c r="A65" s="29" t="s">
-        <v>257</v>
-      </c>
-      <c r="B65" s="33">
+      <c r="A65" s="30" t="s">
+        <v>258</v>
+      </c>
+      <c r="B65" s="34">
         <v>26.91</v>
       </c>
-      <c r="C65" s="33">
+      <c r="C65" s="34">
         <v>22.72</v>
       </c>
-      <c r="D65" s="32"/>
-      <c r="E65" s="33">
+      <c r="D65" s="33"/>
+      <c r="E65" s="34">
         <v>19.02</v>
       </c>
-      <c r="F65" s="33">
+      <c r="F65" s="34">
         <v>16.06</v>
       </c>
-      <c r="G65" s="33">
+      <c r="G65" s="34">
         <v>38.22</v>
       </c>
-      <c r="H65" s="33">
+      <c r="H65" s="34">
         <v>18.21</v>
       </c>
-      <c r="I65" s="33">
+      <c r="I65" s="34">
         <v>9.77</v>
       </c>
-      <c r="J65" s="33">
+      <c r="J65" s="34">
         <v>13.37</v>
       </c>
-      <c r="K65" s="32"/>
-      <c r="L65" s="32"/>
+      <c r="K65" s="33"/>
+      <c r="L65" s="33"/>
     </row>
     <row r="66" ht="15.0" customHeight="1">
-      <c r="A66" s="29" t="s">
-        <v>258</v>
-      </c>
-      <c r="B66" s="33">
+      <c r="A66" s="30" t="s">
+        <v>259</v>
+      </c>
+      <c r="B66" s="34">
         <v>29.52</v>
       </c>
-      <c r="C66" s="33">
+      <c r="C66" s="34">
         <v>30.91</v>
       </c>
-      <c r="D66" s="33">
+      <c r="D66" s="34">
         <v>34.06</v>
       </c>
-      <c r="E66" s="33">
+      <c r="E66" s="34">
         <v>18.14</v>
       </c>
-      <c r="F66" s="33">
+      <c r="F66" s="34">
         <v>16.67</v>
       </c>
-      <c r="G66" s="33">
+      <c r="G66" s="34">
         <v>22.44</v>
       </c>
-      <c r="H66" s="32"/>
-      <c r="I66" s="32"/>
-      <c r="J66" s="32"/>
-      <c r="K66" s="32"/>
-      <c r="L66" s="32"/>
+      <c r="H66" s="33"/>
+      <c r="I66" s="33"/>
+      <c r="J66" s="33"/>
+      <c r="K66" s="33"/>
+      <c r="L66" s="33"/>
     </row>
     <row r="67" ht="15.0" customHeight="1">
-      <c r="A67" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="B67" s="28"/>
-      <c r="C67" s="28"/>
-      <c r="D67" s="28"/>
-      <c r="E67" s="28"/>
-      <c r="F67" s="28"/>
-      <c r="G67" s="28"/>
-      <c r="H67" s="28"/>
-      <c r="I67" s="28"/>
-      <c r="J67" s="28"/>
-      <c r="K67" s="28"/>
-      <c r="L67" s="28"/>
+      <c r="A67" s="28" t="s">
+        <v>260</v>
+      </c>
+      <c r="B67" s="29"/>
+      <c r="C67" s="29"/>
+      <c r="D67" s="29"/>
+      <c r="E67" s="29"/>
+      <c r="F67" s="29"/>
+      <c r="G67" s="29"/>
+      <c r="H67" s="29"/>
+      <c r="I67" s="29"/>
+      <c r="J67" s="29"/>
+      <c r="K67" s="29"/>
+      <c r="L67" s="29"/>
     </row>
     <row r="68" ht="15.0" customHeight="1">
-      <c r="A68" s="29" t="s">
-        <v>260</v>
-      </c>
-      <c r="B68" s="32"/>
-      <c r="C68" s="32"/>
-      <c r="D68" s="32"/>
-      <c r="E68" s="32"/>
-      <c r="F68" s="32"/>
-      <c r="G68" s="32"/>
-      <c r="H68" s="32"/>
-      <c r="I68" s="32"/>
-      <c r="J68" s="32"/>
-      <c r="K68" s="32"/>
-      <c r="L68" s="32"/>
+      <c r="A68" s="30" t="s">
+        <v>261</v>
+      </c>
+      <c r="B68" s="33"/>
+      <c r="C68" s="33"/>
+      <c r="D68" s="33"/>
+      <c r="E68" s="33"/>
+      <c r="F68" s="33"/>
+      <c r="G68" s="33"/>
+      <c r="H68" s="33"/>
+      <c r="I68" s="33"/>
+      <c r="J68" s="33"/>
+      <c r="K68" s="33"/>
+      <c r="L68" s="33"/>
     </row>
     <row r="69" ht="15.75" customHeight="1"/>
     <row r="70" ht="15.75" customHeight="1"/>

</xml_diff>